<commit_message>
last send  by zohair
</commit_message>
<xml_diff>
--- a/New_Ds/production_scheduling/planning_methode1_operateurs_fixes.xlsx
+++ b/New_Ds/production_scheduling/planning_methode1_operateurs_fixes.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planning" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charge par opérateur" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bilan Objectifs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charge par Op et Shift" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charge totale par Op" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bilan Objectifs" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -39,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -52,6 +53,27 @@
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -427,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,7 +480,17 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Priorité EDD</t>
+          <t>Date échéance</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Poids</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Score</t>
         </is>
       </c>
     </row>
@@ -482,8 +514,16 @@
       <c r="E2" t="n">
         <v>3</v>
       </c>
-      <c r="F2" t="n">
-        <v>1</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="3">
@@ -506,8 +546,16 @@
       <c r="E3" t="n">
         <v>2</v>
       </c>
-      <c r="F3" t="n">
-        <v>1</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="4">
@@ -530,8 +578,16 @@
       <c r="E4" t="n">
         <v>2</v>
       </c>
-      <c r="F4" t="n">
-        <v>1</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="5">
@@ -554,8 +610,16 @@
       <c r="E5" t="n">
         <v>1</v>
       </c>
-      <c r="F5" t="n">
-        <v>1</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="6">
@@ -578,8 +642,16 @@
       <c r="E6" t="n">
         <v>3</v>
       </c>
-      <c r="F6" t="n">
-        <v>1</v>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>3</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="7">
@@ -596,14 +668,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>M500325</t>
+          <t>M500304</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F7" t="n">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.263</v>
       </c>
     </row>
     <row r="8">
@@ -615,19 +695,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>OP4</t>
+          <t>OP6</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>M500324</t>
+          <t>M502026</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>8</v>
-      </c>
-      <c r="F8" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>5</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.45</v>
       </c>
     </row>
     <row r="9">
@@ -635,23 +723,31 @@
         <v>1</v>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>OP1</t>
+          <t>OP4</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>M400228</t>
+          <t>M500324</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
-      </c>
-      <c r="F9" t="n">
-        <v>1</v>
+        <v>8</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.513</v>
       </c>
     </row>
     <row r="10">
@@ -663,7 +759,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>OP2</t>
+          <t>OP1</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -672,10 +768,18 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
-      </c>
-      <c r="F10" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="11">
@@ -687,7 +791,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>OP7</t>
+          <t>OP2</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -698,8 +802,16 @@
       <c r="E11" t="n">
         <v>2</v>
       </c>
-      <c r="F11" t="n">
-        <v>1</v>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="12">
@@ -711,7 +823,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>OP8</t>
+          <t>OP7</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -720,10 +832,18 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="13">
@@ -735,7 +855,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>OP10</t>
+          <t>OP8</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -744,10 +864,18 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
-      </c>
-      <c r="F13" t="n">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>3</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="14">
@@ -759,19 +887,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>OP3</t>
+          <t>OP10</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>M500325</t>
+          <t>M400228</t>
         </is>
       </c>
       <c r="E14" t="n">
         <v>3</v>
       </c>
-      <c r="F14" t="n">
-        <v>2</v>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="15">
@@ -783,19 +919,27 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>OP4</t>
+          <t>OP3</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>M500324</t>
+          <t>M500304</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>8</v>
-      </c>
-      <c r="F15" t="n">
-        <v>3</v>
+        <v>5</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>5</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.263</v>
       </c>
     </row>
     <row r="16">
@@ -807,19 +951,27 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>OP6</t>
+          <t>OP4</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>M502026</t>
+          <t>M500324</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" t="n">
-        <v>3</v>
+        <v>8</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>3</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.513</v>
       </c>
     </row>
     <row r="17">
@@ -836,14 +988,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>M500329</t>
+          <t>M500327</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>4</v>
-      </c>
-      <c r="F17" t="n">
-        <v>4</v>
+        <v>3</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>5</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.575</v>
       </c>
     </row>
     <row r="18">
@@ -851,23 +1011,31 @@
         <v>1</v>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>OP1</t>
+          <t>OP9</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>M400228</t>
+          <t>M500327</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
-      </c>
-      <c r="F18" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>5</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.575</v>
       </c>
     </row>
     <row r="19">
@@ -879,7 +1047,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>OP2</t>
+          <t>OP1</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -888,10 +1056,18 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
-      </c>
-      <c r="F19" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>3</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="20">
@@ -903,19 +1079,27 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>OP8</t>
+          <t>OP2</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>M400229</t>
+          <t>M400228</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="21">
@@ -927,19 +1111,27 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>OP10</t>
+          <t>OP7</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>M400229</t>
+          <t>M400200</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>3</v>
-      </c>
-      <c r="F21" t="n">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>5</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.174</v>
       </c>
     </row>
     <row r="22">
@@ -951,7 +1143,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>OP7</t>
+          <t>OP10</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -960,10 +1152,18 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>5</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.174</v>
       </c>
     </row>
     <row r="23">
@@ -975,19 +1175,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>OP3</t>
+          <t>OP8</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>M500325</t>
+          <t>M400229</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>3</v>
-      </c>
-      <c r="F23" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>2</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.225</v>
       </c>
     </row>
     <row r="24">
@@ -999,19 +1207,27 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>OP4</t>
+          <t>OP3</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>M500324</t>
+          <t>M500304</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>8</v>
-      </c>
-      <c r="F24" t="n">
-        <v>3</v>
+        <v>5</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>5</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.263</v>
       </c>
     </row>
     <row r="25">
@@ -1023,19 +1239,27 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>OP5</t>
+          <t>OP4</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>M500327</t>
+          <t>M500324</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F25" t="n">
-        <v>5</v>
+        <v>8</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>3</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.513</v>
       </c>
     </row>
     <row r="26">
@@ -1047,7 +1271,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>OP9</t>
+          <t>OP5</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1056,34 +1280,50 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
-      </c>
-      <c r="F26" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
         <v>5</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.575</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>OP1</t>
+          <t>OP9</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>M400229</t>
+          <t>M500327</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
-      </c>
-      <c r="F27" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>5</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.575</v>
       </c>
     </row>
     <row r="28">
@@ -1095,19 +1335,27 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>OP2</t>
+          <t>OP1</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>M400229</t>
+          <t>M400200</t>
         </is>
       </c>
       <c r="E28" t="n">
         <v>2</v>
       </c>
-      <c r="F28" t="n">
-        <v>1</v>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>5</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.174</v>
       </c>
     </row>
     <row r="29">
@@ -1119,19 +1367,27 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>OP8</t>
+          <t>OP2</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>M400229</t>
+          <t>M400200</t>
         </is>
       </c>
       <c r="E29" t="n">
         <v>1</v>
       </c>
-      <c r="F29" t="n">
-        <v>1</v>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>5</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.174</v>
       </c>
     </row>
     <row r="30">
@@ -1143,19 +1399,27 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>OP10</t>
+          <t>OP7</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>M400229</t>
+          <t>M400200</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>3</v>
-      </c>
-      <c r="F30" t="n">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>5</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.174</v>
       </c>
     </row>
     <row r="31">
@@ -1167,7 +1431,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>OP7</t>
+          <t>OP10</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1176,10 +1440,18 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>5</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.174</v>
       </c>
     </row>
     <row r="32">
@@ -1191,19 +1463,27 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>OP3</t>
+          <t>OP8</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>M500325</t>
+          <t>M400229</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>3</v>
-      </c>
-      <c r="F32" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>2</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.225</v>
       </c>
     </row>
     <row r="33">
@@ -1215,19 +1495,27 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>OP4</t>
+          <t>OP3</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>M500324</t>
+          <t>M500304</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>8</v>
-      </c>
-      <c r="F33" t="n">
-        <v>3</v>
+        <v>5</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>5</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0.263</v>
       </c>
     </row>
     <row r="34">
@@ -1235,23 +1523,31 @@
         <v>2</v>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>OP1</t>
+          <t>OP4</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>M400229</t>
+          <t>M500324</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>3</v>
-      </c>
-      <c r="F34" t="n">
-        <v>1</v>
+        <v>8</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>3</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.513</v>
       </c>
     </row>
     <row r="35">
@@ -1259,23 +1555,31 @@
         <v>2</v>
       </c>
       <c r="B35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>OP2</t>
+          <t>OP5</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>M400229</t>
+          <t>M500327</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>2</v>
-      </c>
-      <c r="F35" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>5</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.575</v>
       </c>
     </row>
     <row r="36">
@@ -1287,19 +1591,27 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>OP8</t>
+          <t>OP1</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>M400229</t>
+          <t>M400200</t>
         </is>
       </c>
       <c r="E36" t="n">
         <v>1</v>
       </c>
-      <c r="F36" t="n">
-        <v>1</v>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>5</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.174</v>
       </c>
     </row>
     <row r="37">
@@ -1311,19 +1623,27 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>OP10</t>
+          <t>OP2</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>M400229</t>
+          <t>M400201</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>3</v>
-      </c>
-      <c r="F37" t="n">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>4</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0.185</v>
       </c>
     </row>
     <row r="38">
@@ -1335,19 +1655,27 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>OP7</t>
+          <t>OP10</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>M400200</t>
+          <t>M400201</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>1</v>
-      </c>
-      <c r="F38" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>4</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.185</v>
       </c>
     </row>
     <row r="39">
@@ -1359,19 +1687,27 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>OP3</t>
+          <t>OP8</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>M500325</t>
+          <t>M400229</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>3</v>
-      </c>
-      <c r="F39" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>2</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.225</v>
       </c>
     </row>
     <row r="40">
@@ -1383,19 +1719,27 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>OP4</t>
+          <t>OP3</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>M500319</t>
+          <t>M500325</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>8</v>
-      </c>
-      <c r="F40" t="n">
-        <v>3</v>
+        <v>3</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>4</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0.328</v>
       </c>
     </row>
     <row r="41">
@@ -1407,19 +1751,27 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>OP5</t>
+          <t>OP7</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>M500327</t>
+          <t>M500325</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>3</v>
-      </c>
-      <c r="F41" t="n">
-        <v>5</v>
+        <v>2</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>4</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.328</v>
       </c>
     </row>
     <row r="42">
@@ -1431,7 +1783,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>OP9</t>
+          <t>OP5</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1440,10 +1792,18 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>2</v>
-      </c>
-      <c r="F42" t="n">
+        <v>3</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
         <v>5</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0.575</v>
       </c>
     </row>
     <row r="43">
@@ -1451,23 +1811,31 @@
         <v>2</v>
       </c>
       <c r="B43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>OP1</t>
+          <t>OP9</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>M400229</t>
+          <t>M500327</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>3</v>
-      </c>
-      <c r="F43" t="n">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>5</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.575</v>
       </c>
     </row>
     <row r="44">
@@ -1475,23 +1843,31 @@
         <v>2</v>
       </c>
       <c r="B44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>OP2</t>
+          <t>OP4</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>M400229</t>
+          <t>M500319</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>2</v>
-      </c>
-      <c r="F44" t="n">
-        <v>1</v>
+        <v>8</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>2</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.613</v>
       </c>
     </row>
     <row r="45">
@@ -1503,7 +1879,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>OP10</t>
+          <t>OP1</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1514,8 +1890,16 @@
       <c r="E45" t="n">
         <v>2</v>
       </c>
-      <c r="F45" t="n">
-        <v>1</v>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>4</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.185</v>
       </c>
     </row>
     <row r="46">
@@ -1527,19 +1911,27 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>OP7</t>
+          <t>OP2</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>M400200</t>
+          <t>M400201</t>
         </is>
       </c>
       <c r="E46" t="n">
         <v>1</v>
       </c>
-      <c r="F46" t="n">
-        <v>1</v>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>4</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.185</v>
       </c>
     </row>
     <row r="47">
@@ -1551,19 +1943,27 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>OP3</t>
+          <t>OP10</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>M500325</t>
+          <t>M400201</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>3</v>
-      </c>
-      <c r="F47" t="n">
-        <v>2</v>
+        <v>2</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>4</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0.185</v>
       </c>
     </row>
     <row r="48">
@@ -1575,19 +1975,27 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>OP4</t>
+          <t>OP8</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>M500319</t>
+          <t>M400229</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>8</v>
-      </c>
-      <c r="F48" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>2</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0.225</v>
       </c>
     </row>
     <row r="49">
@@ -1599,19 +2007,27 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>OP8</t>
+          <t>OP3</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>M500319</t>
+          <t>M500325</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>6</v>
-      </c>
-      <c r="F49" t="n">
-        <v>3</v>
+        <v>3</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>4</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0.328</v>
       </c>
     </row>
     <row r="50">
@@ -1623,19 +2039,27 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>OP5</t>
+          <t>OP7</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>M500327</t>
+          <t>M500325</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>3</v>
-      </c>
-      <c r="F50" t="n">
-        <v>5</v>
+        <v>2</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>4</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0.328</v>
       </c>
     </row>
     <row r="51">
@@ -1647,67 +2071,91 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>OP9</t>
+          <t>OP4</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>M500327</t>
+          <t>M500319</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>2</v>
-      </c>
-      <c r="F51" t="n">
-        <v>5</v>
+        <v>8</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>2</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0.613</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B52" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>OP1</t>
+          <t>OP5</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>M400201</t>
+          <t>M500329</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>2</v>
-      </c>
-      <c r="F52" t="n">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>4</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0.638</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B53" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>OP2</t>
+          <t>OP9</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>M400201</t>
+          <t>M500311</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>1</v>
-      </c>
-      <c r="F53" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>3</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0.77</v>
       </c>
     </row>
     <row r="54">
@@ -1719,7 +2167,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>OP10</t>
+          <t>OP1</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1730,8 +2178,16 @@
       <c r="E54" t="n">
         <v>2</v>
       </c>
-      <c r="F54" t="n">
-        <v>1</v>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>4</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0.185</v>
       </c>
     </row>
     <row r="55">
@@ -1743,19 +2199,27 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>OP7</t>
+          <t>OP2</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>M400200</t>
+          <t>M400201</t>
         </is>
       </c>
       <c r="E55" t="n">
         <v>1</v>
       </c>
-      <c r="F55" t="n">
-        <v>1</v>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>4</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0.185</v>
       </c>
     </row>
     <row r="56">
@@ -1767,19 +2231,27 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>OP3</t>
+          <t>OP10</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>M500325</t>
+          <t>M400201</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>3</v>
-      </c>
-      <c r="F56" t="n">
-        <v>2</v>
+        <v>2</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>4</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0.185</v>
       </c>
     </row>
     <row r="57">
@@ -1791,19 +2263,27 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>OP4</t>
+          <t>OP8</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>M500319</t>
+          <t>M400229</t>
         </is>
       </c>
       <c r="E57" t="n">
         <v>1</v>
       </c>
-      <c r="F57" t="n">
-        <v>3</v>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>2</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0.225</v>
       </c>
     </row>
     <row r="58">
@@ -1815,19 +2295,27 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>OP5</t>
+          <t>OP3</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>M500327</t>
+          <t>M500325</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>2</v>
-      </c>
-      <c r="F58" t="n">
-        <v>5</v>
+        <v>3</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>4</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0.328</v>
       </c>
     </row>
     <row r="59">
@@ -1835,23 +2323,31 @@
         <v>3</v>
       </c>
       <c r="B59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>OP1</t>
+          <t>OP7</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>M400201</t>
+          <t>M500325</t>
         </is>
       </c>
       <c r="E59" t="n">
         <v>2</v>
       </c>
-      <c r="F59" t="n">
-        <v>1</v>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>4</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0.328</v>
       </c>
     </row>
     <row r="60">
@@ -1859,23 +2355,31 @@
         <v>3</v>
       </c>
       <c r="B60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>OP2</t>
+          <t>OP4</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>M400201</t>
+          <t>M500319</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>1</v>
-      </c>
-      <c r="F60" t="n">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>2</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0.613</v>
       </c>
     </row>
     <row r="61">
@@ -1883,23 +2387,31 @@
         <v>3</v>
       </c>
       <c r="B61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>OP10</t>
+          <t>OP5</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>M400201</t>
+          <t>M500311</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>2</v>
-      </c>
-      <c r="F61" t="n">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>3</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0.77</v>
       </c>
     </row>
     <row r="62">
@@ -1911,19 +2423,27 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>OP7</t>
+          <t>OP1</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>M400200</t>
+          <t>M400229</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>1</v>
-      </c>
-      <c r="F62" t="n">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>2</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0.225</v>
       </c>
     </row>
     <row r="63">
@@ -1935,19 +2455,27 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>OP3</t>
+          <t>OP2</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>M500325</t>
+          <t>M400229</t>
         </is>
       </c>
       <c r="E63" t="n">
         <v>2</v>
       </c>
-      <c r="F63" t="n">
-        <v>2</v>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>2</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0.225</v>
       </c>
     </row>
     <row r="64">
@@ -1959,19 +2487,27 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>OP4</t>
+          <t>OP8</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>M500317</t>
+          <t>M400229</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>4</v>
-      </c>
-      <c r="F64" t="n">
-        <v>4</v>
+        <v>1</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>2</v>
+      </c>
+      <c r="H64" t="n">
+        <v>0.225</v>
       </c>
     </row>
     <row r="65">
@@ -1983,19 +2519,27 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>OP5</t>
+          <t>OP10</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>M500311</t>
+          <t>M400229</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>4</v>
-      </c>
-      <c r="F65" t="n">
-        <v>5</v>
+        <v>3</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>2</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0.225</v>
       </c>
     </row>
     <row r="66">
@@ -2007,19 +2551,27 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>OP9</t>
+          <t>OP3</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>M500311</t>
+          <t>M500325</t>
         </is>
       </c>
       <c r="E66" t="n">
         <v>3</v>
       </c>
-      <c r="F66" t="n">
-        <v>5</v>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>4</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0.328</v>
       </c>
     </row>
     <row r="67">
@@ -2027,23 +2579,31 @@
         <v>3</v>
       </c>
       <c r="B67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>OP1</t>
+          <t>OP7</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>M400201</t>
+          <t>M500325</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>1</v>
-      </c>
-      <c r="F67" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>4</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0.328</v>
       </c>
     </row>
     <row r="68">
@@ -2051,23 +2611,31 @@
         <v>3</v>
       </c>
       <c r="B68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>OP2</t>
+          <t>OP5</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>M400200</t>
+          <t>M500311</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>1</v>
-      </c>
-      <c r="F68" t="n">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>3</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0.77</v>
       </c>
     </row>
     <row r="69">
@@ -2075,23 +2643,31 @@
         <v>3</v>
       </c>
       <c r="B69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>OP7</t>
+          <t>OP4</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>M400200</t>
+          <t>M500317</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>1</v>
-      </c>
-      <c r="F69" t="n">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>1</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0.797</v>
       </c>
     </row>
     <row r="70">
@@ -2099,23 +2675,31 @@
         <v>3</v>
       </c>
       <c r="B70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>OP10</t>
+          <t>OP9</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>M400200</t>
+          <t>M500328</t>
         </is>
       </c>
       <c r="E70" t="n">
         <v>2</v>
       </c>
-      <c r="F70" t="n">
-        <v>1</v>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>2</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0.899</v>
       </c>
     </row>
     <row r="71">
@@ -2127,19 +2711,27 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>OP3</t>
+          <t>OP1</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>M500304</t>
+          <t>M400229</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>5</v>
-      </c>
-      <c r="F71" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H71" t="n">
+        <v>0.225</v>
       </c>
     </row>
     <row r="72">
@@ -2151,19 +2743,27 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>OP4</t>
+          <t>OP2</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>M500317</t>
+          <t>M400229</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>4</v>
-      </c>
-      <c r="F72" t="n">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>2</v>
+      </c>
+      <c r="H72" t="n">
+        <v>0.225</v>
       </c>
     </row>
     <row r="73">
@@ -2175,19 +2775,27 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>OP5</t>
+          <t>OP8</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>M500311</t>
+          <t>M400229</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>4</v>
-      </c>
-      <c r="F73" t="n">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>2</v>
+      </c>
+      <c r="H73" t="n">
+        <v>0.225</v>
       </c>
     </row>
     <row r="74">
@@ -2199,51 +2807,67 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>OP9</t>
+          <t>OP10</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>M500328</t>
+          <t>M400229</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>2</v>
-      </c>
-      <c r="F74" t="n">
-        <v>5</v>
+        <v>3</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>2</v>
+      </c>
+      <c r="H74" t="n">
+        <v>0.225</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
+        <v>3</v>
+      </c>
+      <c r="B75" t="n">
+        <v>3</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>OP3</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>M500325</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>3</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
         <v>4</v>
       </c>
-      <c r="B75" t="n">
-        <v>1</v>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>OP3</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>M500304</t>
-        </is>
-      </c>
-      <c r="E75" t="n">
-        <v>5</v>
-      </c>
-      <c r="F75" t="n">
-        <v>2</v>
+      <c r="H75" t="n">
+        <v>0.328</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B76" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2252,86 +2876,118 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>M500304</t>
+          <t>M500309</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>4</v>
-      </c>
-      <c r="F76" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>1</v>
+      </c>
+      <c r="H76" t="n">
+        <v>0.624</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
+        <v>3</v>
+      </c>
+      <c r="B77" t="n">
+        <v>3</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>OP4</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>M500317</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
         <v>4</v>
       </c>
-      <c r="B77" t="n">
-        <v>1</v>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>OP10</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>M500304</t>
-        </is>
-      </c>
-      <c r="E77" t="n">
-        <v>6</v>
-      </c>
-      <c r="F77" t="n">
-        <v>2</v>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>1</v>
+      </c>
+      <c r="H77" t="n">
+        <v>0.797</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B78" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>OP2</t>
+          <t>OP5</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>M500309</t>
+          <t>M500328</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>1</v>
-      </c>
-      <c r="F78" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>2</v>
+      </c>
+      <c r="H78" t="n">
+        <v>0.899</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>OP4</t>
+          <t>OP9</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>M500317</t>
+          <t>M500328</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>4</v>
-      </c>
-      <c r="F79" t="n">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
+        <v>2</v>
+      </c>
+      <c r="H79" t="n">
+        <v>0.899</v>
       </c>
     </row>
     <row r="80">
@@ -2343,19 +2999,27 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>OP5</t>
+          <t>OP1</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>M500328</t>
+          <t>M400229</t>
         </is>
       </c>
       <c r="E80" t="n">
         <v>3</v>
       </c>
-      <c r="F80" t="n">
-        <v>5</v>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
+        <v>2</v>
+      </c>
+      <c r="H80" t="n">
+        <v>0.225</v>
       </c>
     </row>
     <row r="81">
@@ -2367,19 +3031,27 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>OP9</t>
+          <t>OP2</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>M500328</t>
+          <t>M400229</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>2</v>
-      </c>
-      <c r="F81" t="n">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>2</v>
+      </c>
+      <c r="H81" t="n">
+        <v>0.225</v>
       </c>
     </row>
     <row r="82">
@@ -2387,7 +3059,7 @@
         <v>4</v>
       </c>
       <c r="B82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -2402,8 +3074,16 @@
       <c r="E82" t="n">
         <v>4</v>
       </c>
-      <c r="F82" t="n">
-        <v>4</v>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="G82" t="n">
+        <v>1</v>
+      </c>
+      <c r="H82" t="n">
+        <v>0.797</v>
       </c>
     </row>
     <row r="83">
@@ -2411,7 +3091,7 @@
         <v>4</v>
       </c>
       <c r="B83" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2426,8 +3106,16 @@
       <c r="E83" t="n">
         <v>5</v>
       </c>
-      <c r="F83" t="n">
-        <v>4</v>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="G83" t="n">
+        <v>1</v>
+      </c>
+      <c r="H83" t="n">
+        <v>0.797</v>
       </c>
     </row>
     <row r="84">
@@ -2435,7 +3123,7 @@
         <v>4</v>
       </c>
       <c r="B84" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2450,8 +3138,16 @@
       <c r="E84" t="n">
         <v>2</v>
       </c>
-      <c r="F84" t="n">
-        <v>5</v>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="G84" t="n">
+        <v>2</v>
+      </c>
+      <c r="H84" t="n">
+        <v>0.899</v>
       </c>
     </row>
     <row r="85">
@@ -2459,7 +3155,7 @@
         <v>4</v>
       </c>
       <c r="B85" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2474,8 +3170,48 @@
       <c r="E85" t="n">
         <v>4</v>
       </c>
-      <c r="F85" t="n">
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="G85" t="n">
+        <v>1</v>
+      </c>
+      <c r="H85" t="n">
+        <v>0.797</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
         <v>4</v>
+      </c>
+      <c r="B86" t="n">
+        <v>2</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>OP10</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>M500317</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>4</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="G86" t="n">
+        <v>1</v>
+      </c>
+      <c r="H86" t="n">
+        <v>0.797</v>
       </c>
     </row>
   </sheetData>
@@ -2489,7 +3225,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2500,10 +3236,15 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Quantité</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Nombre de shifts</t>
         </is>
@@ -2515,131 +3256,376 @@
           <t>OP1</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>23</v>
+      <c r="B2" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="D2" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>OP10</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>34</v>
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="n">
+        <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>11</v>
+        <v>7</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>OP2</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>16</v>
+      <c r="A4" s="1" t="n"/>
+      <c r="B4" s="1" t="n">
+        <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>OP3</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>33</v>
+          <t>OP10</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>10</v>
+        <v>12</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>OP4</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>69</v>
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="1" t="n">
+        <v>2</v>
       </c>
       <c r="C6" t="n">
         <v>12</v>
       </c>
+      <c r="D6" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>OP5</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>28</v>
+      <c r="A7" s="1" t="n"/>
+      <c r="B7" s="1" t="n">
+        <v>3</v>
       </c>
       <c r="C7" t="n">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>OP6</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+          <t>OP2</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="D8" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>OP7</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>15</v>
+      <c r="A9" s="1" t="n"/>
+      <c r="B9" s="1" t="n">
+        <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>10</v>
+        <v>5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>OP8</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>11</v>
+      <c r="A10" s="1" t="n"/>
+      <c r="B10" s="1" t="n">
+        <v>3</v>
       </c>
       <c r="C10" t="n">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
+          <t>OP3</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>13</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n"/>
+      <c r="B12" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" t="n">
+        <v>11</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n"/>
+      <c r="B13" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" t="n">
+        <v>11</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>OP4</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>27</v>
+      </c>
+      <c r="D14" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n"/>
+      <c r="B15" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="n">
+        <v>24</v>
+      </c>
+      <c r="D15" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n"/>
+      <c r="B16" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="n">
+        <v>20</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>OP5</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="n">
+        <v>9</v>
+      </c>
+      <c r="D17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n"/>
+      <c r="B18" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n"/>
+      <c r="B19" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="n">
+        <v>10</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>OP6</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>OP7</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" t="n">
+        <v>5</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n"/>
+      <c r="B22" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" t="n">
+        <v>6</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n"/>
+      <c r="B23" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" t="n">
+        <v>4</v>
+      </c>
+      <c r="D23" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>OP8</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n"/>
+      <c r="B25" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n"/>
+      <c r="B26" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
           <t>OP9</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>13</v>
-      </c>
-      <c r="C11" t="n">
-        <v>6</v>
+      <c r="B27" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" t="n">
+        <v>5</v>
+      </c>
+      <c r="D27" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n"/>
+      <c r="B28" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" t="n">
+        <v>7</v>
+      </c>
+      <c r="D28" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A24:A26"/>
+    <mergeCell ref="A14:A16"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2650,6 +3636,167 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Opérateur</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Quantité</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Nombre de shifts</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>OP1</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>25</v>
+      </c>
+      <c r="C2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>OP10</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>31</v>
+      </c>
+      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>OP2</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>15</v>
+      </c>
+      <c r="C4" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>OP3</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>35</v>
+      </c>
+      <c r="C5" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>OP4</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>71</v>
+      </c>
+      <c r="C6" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>OP5</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>29</v>
+      </c>
+      <c r="C7" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>OP6</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>OP7</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>15</v>
+      </c>
+      <c r="C9" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>OP8</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>OP9</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>12</v>
+      </c>
+      <c r="C11" t="n">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>